<commit_message>
Made headway on chlorophyll report.
</commit_message>
<xml_diff>
--- a/files/cali_summary_2022-07_29_new_modules.xlsx
+++ b/files/cali_summary_2022-07_29_new_modules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\justin.belluz\Documents\R\chl_qc\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4912472-8A21-4DB4-B596-1775A8C82016}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F966C5B1-6F72-46BB-93D4-960A8370B73A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="14604" activeTab="1" xr2:uid="{58D8BF88-922C-47DB-AA1D-0750D9F9DE65}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="14604" xr2:uid="{58D8BF88-922C-47DB-AA1D-0750D9F9DE65}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
   <si>
     <t>Date</t>
   </si>
@@ -465,7 +465,7 @@
   <cols>
     <col min="1" max="1" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="11.109375" customWidth="1"/>
     <col min="6" max="6" width="8.88671875" style="3"/>
     <col min="7" max="7" width="12" style="4" bestFit="1" customWidth="1"/>
@@ -662,19 +662,58 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="11"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="15"/>
+      <c r="A8" s="11">
+        <v>45511</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8">
+        <v>720001154</v>
+      </c>
+      <c r="D8" s="12">
+        <v>97295.57</v>
+      </c>
+      <c r="E8" s="12">
+        <v>100723.82</v>
+      </c>
+      <c r="F8" s="13">
+        <v>1.75</v>
+      </c>
+      <c r="G8" s="14">
+        <v>4.6835686149999999E-4</v>
+      </c>
+      <c r="H8" s="15">
+        <v>0.99986112380000003</v>
+      </c>
       <c r="I8" s="11"/>
       <c r="J8" s="12"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="A9" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9">
+        <v>720000982</v>
+      </c>
+      <c r="D9" s="5">
+        <v>73165.97</v>
+      </c>
+      <c r="E9" s="5">
+        <v>80487.28</v>
+      </c>
+      <c r="F9" s="3">
+        <v>1.76</v>
+      </c>
+      <c r="G9" s="4">
+        <v>3.5645310439999999E-4</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0.99987826020000004</v>
+      </c>
       <c r="I9" s="11"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -715,7 +754,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{297A9660-58AB-44EA-B3B6-7AC55341B8F5}">
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -1534,6 +1573,272 @@
         <v>1.7147182650373909</v>
       </c>
     </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B50">
+        <v>720001154</v>
+      </c>
+      <c r="C50">
+        <v>0</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B51">
+        <v>720001154</v>
+      </c>
+      <c r="C51">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="D51">
+        <v>4316.9799999999996</v>
+      </c>
+      <c r="E51">
+        <v>1.73</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B52">
+        <v>720001154</v>
+      </c>
+      <c r="C52">
+        <v>10.27</v>
+      </c>
+      <c r="D52">
+        <v>21080.240000000002</v>
+      </c>
+      <c r="E52">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B53">
+        <v>720001154</v>
+      </c>
+      <c r="C53">
+        <v>25.66</v>
+      </c>
+      <c r="D53">
+        <v>53465.98</v>
+      </c>
+      <c r="E53">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B54">
+        <v>720001154</v>
+      </c>
+      <c r="C54">
+        <v>50.64</v>
+      </c>
+      <c r="D54">
+        <v>106944.97</v>
+      </c>
+      <c r="E54">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B55">
+        <v>720001154</v>
+      </c>
+      <c r="C55">
+        <v>75.97</v>
+      </c>
+      <c r="D55">
+        <v>160323.29999999999</v>
+      </c>
+      <c r="E55">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B56">
+        <v>720001154</v>
+      </c>
+      <c r="C56">
+        <v>151.93</v>
+      </c>
+      <c r="D56">
+        <v>317147.94</v>
+      </c>
+      <c r="E56">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B57">
+        <v>720001154</v>
+      </c>
+      <c r="C57">
+        <v>297.54000000000002</v>
+      </c>
+      <c r="D57">
+        <v>636355.31999999995</v>
+      </c>
+      <c r="E57">
+        <v>1.79</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A58" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B58">
+        <v>720000982</v>
+      </c>
+      <c r="C58">
+        <v>0</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B59">
+        <v>720000982</v>
+      </c>
+      <c r="C59">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="D59">
+        <v>5604.74</v>
+      </c>
+      <c r="E59">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A60" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B60">
+        <v>720000982</v>
+      </c>
+      <c r="C60">
+        <v>10.27</v>
+      </c>
+      <c r="D60">
+        <v>27662.48</v>
+      </c>
+      <c r="E60">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B61">
+        <v>720000982</v>
+      </c>
+      <c r="C61">
+        <v>25.66</v>
+      </c>
+      <c r="D61">
+        <v>67734.759999999995</v>
+      </c>
+      <c r="E61">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A62" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B62">
+        <v>720000982</v>
+      </c>
+      <c r="C62">
+        <v>50.64</v>
+      </c>
+      <c r="D62">
+        <v>136618.94</v>
+      </c>
+      <c r="E62">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B63">
+        <v>720000982</v>
+      </c>
+      <c r="C63">
+        <v>75.97</v>
+      </c>
+      <c r="D63">
+        <v>208023.75</v>
+      </c>
+      <c r="E63">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A64" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B64">
+        <v>720000982</v>
+      </c>
+      <c r="C64">
+        <v>151.93</v>
+      </c>
+      <c r="D64">
+        <v>417215.74</v>
+      </c>
+      <c r="E64">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
+        <v>45511</v>
+      </c>
+      <c r="B65">
+        <v>720000982</v>
+      </c>
+      <c r="C65">
+        <v>297.54000000000002</v>
+      </c>
+      <c r="D65">
+        <v>834370.36</v>
+      </c>
+      <c r="E65">
+        <v>1.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>